<commit_message>
docs(snx-20): map LJ calling sheet notes and contact
</commit_message>
<xml_diff>
--- a/docs/contracts/fixtures/synthetic-lead-import-v1.xlsx
+++ b/docs/contracts/fixtures/synthetic-lead-import-v1.xlsx
@@ -172,6 +172,16 @@
           <t>Sample City</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Asked for a follow-up email</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Sam Example</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>

<commit_message>
docs(snx-28): correct the Jacks column mapping from the observed data
The Jacks header row (Facility, Name, Email, Status, ...) does not describe
its data. A counts-only profile of the private workbook, printing no cell
values, showed the data rows use the Ljs A-G layout: A matches Ljs regions
(13 distinct values, 57% shared), E holds every email, C holds the clinic
names. Mapped by header, 585 of 587 rows failed email validation and region
names would have become clinic names.

The contract now records the inferred mapping, the evidence and the need
for SolTech confirmation before a production import. B is no longer held as
unconfirmed evidence; J and K still are. The synthetic fixture uses the
observed layout and stages identically to the importer tests' workbook.
</commit_message>
<xml_diff>
--- a/docs/contracts/fixtures/synthetic-lead-import-v1.xlsx
+++ b/docs/contracts/fixtures/synthetic-lead-import-v1.xlsx
@@ -56,22 +56,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Region Sample</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Province Sample</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Harborview Clinic</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Sam Example</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0917 000 0199</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>harborview@example.test</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0917 000 0199</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sample Street</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sample City</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -98,10 +113,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Region Sample</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>missing-facility@example.test</t>
         </is>
@@ -115,17 +135,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Region Sample</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Pinecrest Clinic</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0917 000 0202</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>pinecrest@example.test</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0917 000 0202</t>
         </is>
       </c>
     </row>

</xml_diff>